<commit_message>
Auto-regenerate festival files from schedule.json
</commit_message>
<xml_diff>
--- a/LaRoche2026_Festival_Schedule.xlsx
+++ b/LaRoche2026_Festival_Schedule.xlsx
@@ -1,17 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Stage" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day Stage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Street Festival" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teaching Camp" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Google Calendar Import" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Main Stage" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Day Stage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Street Festival" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Teaching Camp" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,14 +75,8 @@
       <color rgb="00B7950B"/>
       <sz val="9"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="15">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -150,11 +143,6 @@
         <fgColor rgb="00EAD5F5"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="008B0000"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -182,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -243,15 +231,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -641,7 +620,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill in Start Time and End Time after consulting the schedule image on the festival website</t>
+          <t>Source data: data/schedule.json in the GitHub repository</t>
         </is>
       </c>
     </row>
@@ -715,7 +694,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Times in 24hr format — e.g. 19:00 to 20:00</t>
+          <t>Times in 24hr format</t>
         </is>
       </c>
     </row>
@@ -752,7 +731,7 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>End of teaching camp — students take the stage</t>
+          <t>Teaching camp students perform. Instructors: Kristy Cox, Jason Bailey, Carter Lester, Ellie Hakanson, Tyler Griffith, Ondra Kozák, Raphael Maillet, Patrick Peillon, Dorian Ricaux, Thierry Loyer, Christian Labonne, Marie Clemence, Gilles Rézard</t>
         </is>
       </c>
     </row>
@@ -789,7 +768,7 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Traditional Bluegrass with humour; luthier-led band</t>
+          <t>Traditional Bluegrass with humour; luthier-led band. Band members TBC.</t>
         </is>
       </c>
     </row>
@@ -855,7 +834,7 @@
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>European pioneers; Paul Von Vlodrop on mandolin</t>
+          <t>Paul Von Vlodrop (mandolin), Lluís Gómez (banjo), Maribel Rivero (bass), Jorge Rodriguez Cros (guitar), Noah Hassler-Forest (fiddle)</t>
         </is>
       </c>
     </row>
@@ -887,12 +866,12 @@
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>Nashville-based; 5 studio albums; returning since 2014</t>
+          <t>Kristy Cox (guitar), Ellie Hakanson (fiddle), Jason Bailey (mandolin), Carter Lester (banjo), Tyler Griffith (bass)</t>
         </is>
       </c>
     </row>
@@ -929,7 +908,7 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Rotterdam contest winners; jazz &amp; world music-infused Bluegrass</t>
+          <t>Noah Hassler-Forest (fiddle), Thijs Vrolijk (guitar), Joshua ten Doornkaat (mandolin), Maribel Rivero (bass), Lluís Gómez (banjo)</t>
         </is>
       </c>
     </row>
@@ -966,7 +945,7 @@
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>All-female European supergroup; La Roche debut as full band</t>
+          <t>Signe Borch (guitar, DK), Kylie Kay Anderson (mandolin, US), Loes van Schaijk (bass, NL), Simona Uhereková (banjo, SK), Esther Duerinck (fiddle, BE)</t>
         </is>
       </c>
     </row>
@@ -1003,7 +982,7 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Ondra Kozák; 4-time La Roche contest winners; 10th anniversary</t>
+          <t>Ondra Kozák (guitar/fiddle), Pavel Tim Duda (bass/guitar), Vít Hanulík (mandolin/guitar), Karel Začal (dobro), David Benda (banjo)</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1019,7 @@
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>East Nashville; Sierra Ferrell's touring band</t>
+          <t>Joshua Rilko (mandolin), Oliver Bates Craven (fiddle), Geoff Saunders (bass), Jacob Groopman (guitar), George Guthrie (banjo)</t>
         </is>
       </c>
     </row>
@@ -1072,12 +1051,12 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Montreal; Bluegrass in English and French</t>
+          <t>Léandre Joly-Pelletier (mandolin), Catherine-Audrey Lachapelle (guitar), Jean-Philippe Demers-Lelotte (bass), Kieran Poile (fiddle)</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1093,7 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Berlin-based; Americana/Bluegrass/folk; promoted from Day Stage</t>
+          <t>Jason Serious (guitar), David Stewart Ingleton (banjo), Tomás Peralta (mandolin/banjo/bass/dobro)</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1130,7 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>Young California trio; Berklee scholars; CBA stable</t>
+          <t>Lucy Khadder (fiddle/guitar), Sophia Sparks (mandolin/guitar), Clare O'Grady (bass)</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1167,7 @@
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>Korean Bluegrass; IBMA grant recipients; Grand Ole Opry veterans</t>
+          <t>Jongsu Yoon (fiddle), Yebin Kim (mandolin), Sunjae Won (guitar), Ki Ha (bass), Hyun Ho (banjo)</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1204,7 @@
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>2x Grammy winner (ex-Molly Tuttle); solo album 2025</t>
+          <t>Shelby Means (bass), Joel Timmons (guitar), Jacob Means (mandolin), Ellie Hakanson (fiddle), George Guthrie (banjo)</t>
         </is>
       </c>
     </row>
@@ -1257,12 +1236,12 @@
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>30-year-old band; La Roche contest winners 2008; first visit in 10 years</t>
+          <t>Jaromír Jahoda (banjo), Zdeněk Jahoda (mandolin), Jindřich Vinkler (guitar), Erik Banič (bass)</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1278,7 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Solo cello; classically trained; Chris Thile &amp; Tony Rice influences</t>
+          <t>William Jack (cello). Solo performer; classically trained in Austria.</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1315,7 @@
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>Promoted from Day Stage 2024; Bluegrass/Old Time/Folk mix</t>
+          <t>Abbey Thomas (mandolin), Holly Wheeldon (fiddle/guitar), Ruth Eliza (clawhammer banjo), Esther Duerinck (fiddle), Noémie Charmetant (bass)</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1352,7 @@
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>Celtic-Americana fusion; 3 banjo players incl. Enda Scahill (We Banjo Three)</t>
+          <t>Jacob Ventura (guitar/bass), Lorenzo Testa (tenor banjo/mandolin), Joan Gatti (fiddle), Enda Scahill (tenor banjo), Eric Long (clawhammer banjo)</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1389,7 @@
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
-          <t>2x IBMA Momentum nominees 2022; touring US regulars</t>
+          <t>Rebekka Nilsson (vocals), Ole Enggrav (guitar), Moa Meinich (fiddle), David Buverud (bass), Emil Brattested (dobro/mandolin), Sjur Marqvardsen (accordion)</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1426,7 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Folk-Americana; Paul Simon/Gram Parsons influences; festival closer</t>
+          <t>Jorieke de Vet (cello), Ronald de Jong (bass), Marc Mosmans (acoustic guitar), Pauline de Vet (fiddle), Roger Verbeek (drums), Frans Pruis (lead guitar)</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1468,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill in Start Time and End Time after consulting the schedule image on the festival website</t>
+          <t>Source data: data/schedule.json in the GitHub repository</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1542,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Times in 24hr format — e.g. 19:00 to 20:00</t>
+          <t>Times in 24hr format</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1579,7 @@
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>Ages 6-16; two mornings of workshops culminating in performance</t>
+          <t>Ages 6-16 workshop performance. Instructors: Ti'Pierre Chalfoun, Thomas Marinello, Marie Scheid</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1616,7 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Also headlining Thu Main Stage; second chance to see them</t>
+          <t>Kristy Cox (guitar), Ellie Hakanson (fiddle), Jason Bailey (mandolin), Carter Lester (banjo), Tyler Griffith (bass)</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1653,7 @@
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>Local Alps trio; traditional Bluegrass + modern pop covers</t>
+          <t>Adrien Garlin (guitar), Laurent Chicoisne (banjo/guitar), Dorian Ricaux (mandolin), Michael Clement (bass)</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1690,7 @@
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>Also on Main Stage Fri; Sierra Ferrell's touring band</t>
+          <t>Joshua Rilko (mandolin), Oliver Bates Craven (fiddle), Geoff Saunders (bass), Jacob Groopman (guitar), George Guthrie (banjo)</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1727,7 @@
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>Irishman in Aix-les-Bains; folk/Irish/blues/rock trio</t>
+          <t>Tim O'Connor (guitar), Bertrand Denechaud (dobro), Dave Thom (mandolin/guitar)</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1764,7 @@
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Twin fiddles; folk/country; formed in UK</t>
+          <t>Grace Honeywell (fiddle/guitar), Jeri Foreman (fiddle/guitar)</t>
         </is>
       </c>
     </row>
@@ -1822,7 +1801,7 @@
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>Toulouse veterans; Dawgrass style; mandocello &amp; cello</t>
+          <t>Patrick Portales (guitar/fiddle), Daniel Portales (mandolin/mandocello), Hannah Al-Kharusy (cello)</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1838,7 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Also on Sat Main Stage; entirely different set</t>
+          <t>Shelby Means (bass), Joel Timmons (guitar), Jacob Means (mandolin), Ellie Hakanson (fiddle)</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1875,7 @@
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>Also on Sat Main Stage; final chance before they fly home</t>
+          <t>Jongsu Yoon (fiddle), Yebin Kim (mandolin), Sunjae Won (guitar), Ki Ha (bass), Hyun Ho (banjo)</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1912,7 @@
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Also on Sat Main Stage; California trio</t>
+          <t>Lucy Khadder (fiddle/guitar), Sophia Sparks (mandolin), Clare O'Grady (bass)</t>
         </is>
       </c>
     </row>
@@ -1975,7 +1954,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill in Start Time and End Time after consulting the schedule image on the festival website</t>
+          <t>Source data: data/schedule.json in the GitHub repository</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2028,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Times in 24hr format — e.g. 19:00 to 20:00</t>
+          <t>Times in 24hr format</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2057,7 @@
       <c r="F5" s="17" t="inlineStr"/>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
+          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2086,7 @@
       <c r="F6" s="17" t="inlineStr"/>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
+          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2115,7 @@
       <c r="F7" s="17" t="inlineStr"/>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
+          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
         </is>
       </c>
     </row>
@@ -2165,7 +2144,7 @@
       <c r="F8" s="17" t="inlineStr"/>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
+          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2173,7 @@
       <c r="F9" s="17" t="inlineStr"/>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
+          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
         </is>
       </c>
     </row>
@@ -2223,7 +2202,7 @@
       <c r="F10" s="17" t="inlineStr"/>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
+          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2231,7 @@
       <c r="F11" s="17" t="inlineStr"/>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>Health centre concert. FREE. Venue &amp; band TBC — check festival website.</t>
+          <t>Health centre concert. FREE. Venue &amp; band TBC.</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2260,7 @@
       <c r="F12" s="17" t="inlineStr"/>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
+          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2289,7 @@
       <c r="F13" s="17" t="inlineStr"/>
       <c r="G13" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
+          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
         </is>
       </c>
     </row>
@@ -2339,7 +2318,7 @@
       <c r="F14" s="17" t="inlineStr"/>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
+          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
         </is>
       </c>
     </row>
@@ -2368,7 +2347,7 @@
       <c r="F15" s="17" t="inlineStr"/>
       <c r="G15" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
+          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
         </is>
       </c>
     </row>
@@ -2397,7 +2376,7 @@
       <c r="F16" s="17" t="inlineStr"/>
       <c r="G16" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
+          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2405,7 @@
       <c r="F17" s="17" t="inlineStr"/>
       <c r="G17" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
+          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
         </is>
       </c>
     </row>
@@ -2455,7 +2434,7 @@
       <c r="F18" s="17" t="inlineStr"/>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>Health centre concert. FREE. Venue &amp; band TBC — check festival website.</t>
+          <t>Health centre concert. FREE. Venue &amp; band TBC.</t>
         </is>
       </c>
     </row>
@@ -2484,7 +2463,7 @@
       <c r="F19" s="17" t="inlineStr"/>
       <c r="G19" s="16" t="inlineStr">
         <is>
-          <t>Health centre concert. FREE. Venue &amp; band TBC — check festival website.</t>
+          <t>Health centre concert. FREE. Venue &amp; band TBC.</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2505,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill in Start Time and End Time after consulting the schedule image on the festival website</t>
+          <t>Source data: data/schedule.json in the GitHub repository</t>
         </is>
       </c>
     </row>
@@ -2600,7 +2579,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Times in 24hr format — e.g. 19:00 to 20:00</t>
+          <t>Times in 24hr format</t>
         </is>
       </c>
     </row>
@@ -2622,15 +2601,20 @@
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="E5" s="20" t="inlineStr">
+      <c r="F5" s="20" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="F5" s="20" t="inlineStr">
+      <c r="G5" s="19" t="inlineStr">
         <is>
           <t>School open for registration and room check-in</t>
         </is>
@@ -2654,15 +2638,20 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>20:00</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>Welcome by Festival Chair and Camp Leader Gilles Rézard</t>
         </is>
@@ -2686,15 +2675,24 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
           <t>20:00</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr"/>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>Welcome dinner</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
@@ -2714,15 +2712,20 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
           <t>07:45</t>
         </is>
       </c>
-      <c r="E8" s="20" t="inlineStr">
+      <c r="F8" s="20" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F8" s="20" t="inlineStr"/>
+      <c r="G8" s="19" t="inlineStr"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -2742,17 +2745,22 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr">
-        <is>
-          <t>Morning session 1 — instrumental classes</t>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Morning session 1</t>
         </is>
       </c>
     </row>
@@ -2774,15 +2782,20 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr"/>
+      <c r="G10" s="8" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -2802,17 +2815,22 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F11" s="11" t="inlineStr">
-        <is>
-          <t>Morning session 2 — instrumental classes</t>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>Morning session 2</t>
         </is>
       </c>
     </row>
@@ -2834,15 +2852,20 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr"/>
+      <c r="G12" s="8" t="inlineStr"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -2862,17 +2885,22 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F13" s="11" t="inlineStr">
-        <is>
-          <t>Afternoon — Wernick Method jam instructions</t>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>Introduction to the Wernick Method coached jam format</t>
         </is>
       </c>
     </row>
@@ -2894,15 +2922,20 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr"/>
+      <c r="G14" s="8" t="inlineStr"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -2922,17 +2955,22 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="F15" s="11" t="inlineStr">
-        <is>
-          <t>Requested/optional modules</t>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>Participant-requested workshop modules</t>
         </is>
       </c>
     </row>
@@ -2954,15 +2992,20 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr"/>
+      <c r="G16" s="8" t="inlineStr"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="19" t="inlineStr">
@@ -2982,15 +3025,20 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
           <t>07:45</t>
         </is>
       </c>
-      <c r="E17" s="20" t="inlineStr">
+      <c r="F17" s="20" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F17" s="20" t="inlineStr"/>
+      <c r="G17" s="19" t="inlineStr"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -3010,17 +3058,22 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t>Morning session 1 — instrumental classes</t>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Morning session 1</t>
         </is>
       </c>
     </row>
@@ -3042,15 +3095,20 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="F19" s="11" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr"/>
+      <c r="G19" s="10" t="inlineStr"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -3070,17 +3128,22 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
-        <is>
-          <t>Morning session 2 — instrumental classes</t>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Morning session 2</t>
         </is>
       </c>
     </row>
@@ -3102,15 +3165,20 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="F21" s="11" t="inlineStr"/>
+      <c r="G21" s="10" t="inlineStr"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -3130,17 +3198,22 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>Afternoon — coached Wernick Method jam</t>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Coached Wernick Method jam</t>
         </is>
       </c>
     </row>
@@ -3162,15 +3235,20 @@
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="F23" s="11" t="inlineStr">
         <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="F23" s="11" t="inlineStr"/>
+      <c r="G23" s="10" t="inlineStr"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -3190,15 +3268,20 @@
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="G24" s="8" t="inlineStr">
         <is>
           <t>Rehearsal for Thursday student concert</t>
         </is>
@@ -3222,15 +3305,20 @@
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="F25" s="11" t="inlineStr">
         <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="F25" s="11" t="inlineStr"/>
+      <c r="G25" s="10" t="inlineStr"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="19" t="inlineStr">
@@ -3250,15 +3338,20 @@
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
           <t>07:45</t>
         </is>
       </c>
-      <c r="E26" s="20" t="inlineStr">
+      <c r="F26" s="20" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F26" s="20" t="inlineStr"/>
+      <c r="G26" s="19" t="inlineStr"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
@@ -3278,17 +3371,22 @@
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="F27" s="11" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F27" s="11" t="inlineStr">
-        <is>
-          <t>Morning session 1 — instrumental classes</t>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>Morning session 1</t>
         </is>
       </c>
     </row>
@@ -3310,15 +3408,20 @@
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="F28" s="9" t="inlineStr"/>
+      <c r="G28" s="8" t="inlineStr"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
@@ -3338,17 +3441,22 @@
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="F29" s="11" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F29" s="11" t="inlineStr">
-        <is>
-          <t>Final morning session — band labs and jams</t>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>Final session before student concert</t>
         </is>
       </c>
     </row>
@@ -3370,15 +3478,20 @@
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="F30" s="9" t="inlineStr"/>
+      <c r="G30" s="8" t="inlineStr"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
@@ -3398,15 +3511,20 @@
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="F31" s="11" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F31" s="11" t="inlineStr"/>
+      <c r="G31" s="10" t="inlineStr"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="8" t="inlineStr">
@@ -3426,15 +3544,20 @@
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="E32" s="9" t="inlineStr">
+      <c r="F32" s="9" t="inlineStr">
         <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="F32" s="9" t="inlineStr"/>
+      <c r="G32" s="8" t="inlineStr"/>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
@@ -3454,17 +3577,22 @@
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="F33" s="11" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="F33" s="11" t="inlineStr">
-        <is>
-          <t>Move to Lycée Sainte Marie festival site</t>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>Travel to Lycée Sainte Marie festival site</t>
         </is>
       </c>
     </row>
@@ -3486,17 +3614,22 @@
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="E34" s="9" t="inlineStr">
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="F34" s="9" t="inlineStr">
-        <is>
-          <t>Band Labs perform on the Main Stage</t>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Band Labs groups perform on the Main Stage</t>
         </is>
       </c>
     </row>
@@ -3518,17 +3651,22 @@
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
+          <t>Teaching Camp</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="F35" s="11" t="inlineStr">
         <is>
           <t>20:00</t>
         </is>
       </c>
-      <c r="F35" s="11" t="inlineStr">
-        <is>
-          <t>French teachers perform on the Main Stage</t>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>French teaching staff perform on the Main Stage</t>
         </is>
       </c>
     </row>
@@ -3539,2197 +3677,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="008B0000"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F79"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>Google Calendar Import — fill in times, then export this sheet as CSV and import into Google Calendar</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="22" t="inlineStr">
-        <is>
-          <t>TBC rows are placeholders for the Street Festival — update when the festival publishes the full street programme</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="23" t="inlineStr">
-        <is>
-          <t>Subject</t>
-        </is>
-      </c>
-      <c r="B3" s="23" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="C3" s="23" t="inlineStr">
-        <is>
-          <t>Start Time</t>
-        </is>
-      </c>
-      <c r="D3" s="23" t="inlineStr">
-        <is>
-          <t>End Date</t>
-        </is>
-      </c>
-      <c r="E3" s="23" t="inlineStr">
-        <is>
-          <t>End Time</t>
-        </is>
-      </c>
-      <c r="F3" s="23" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>Workshop Students &amp; Teachers (Europe) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>End of teaching camp — students take the stage</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>Piotr Bulas &amp; Garage Folks (PL) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>20:45</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>Traditional Bluegrass with humour; luthier-led band</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>Opening Ceremony () — Main Stage</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>20:45</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>21:15</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr"/>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>Paul &amp; The Alley Cats (NL/ES) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>21:15</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>22:45</t>
-        </is>
-      </c>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>European pioneers; Paul Von Vlodrop on mandolin</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>Kristy Cox Band (AU/US) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>22:45</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>01:00</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Nashville-based; 5 studio albums; returning since 2014</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>Noah Hassler-Forest (NL/ES) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>Rotterdam contest winners; jazz &amp; world music-infused Bluegrass</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>No Man's Land (SK/US/NL/DK/BE) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>All-female European supergroup; La Roche debut as full band</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>The New Aliquot &amp; David Benda (CZ) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Ondra Kozák; 4-time La Roche contest winners; 10th anniversary</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>Sentimental Gentlemen (US) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>East Nashville; Sierra Ferrell's touring band</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>Veranda (CA) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>Montreal; Bluegrass in English and French</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Yonder Boys (DE/US/AU/CL) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Berlin-based; Americana/Bluegrass/folk; promoted from Day Stage</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>Sweet Sally (US) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>Young California trio; Berklee scholars; CBA stable</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>Country Gongbang (KO) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>Korean Bluegrass; IBMA grant recipients; Grand Ole Opry veterans</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>Shelby Means Band (US) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="E17" s="10" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
-      <c r="F17" s="10" t="inlineStr">
-        <is>
-          <t>2x Grammy winner (ex-Molly Tuttle); solo album 2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>Monogram (CZ) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>30-year-old band; La Roche contest winners 2008; first visit in 10 years</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>William Jack (AU) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>Solo cello; classically trained; Chris Thile &amp; Tony Rice influences</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>Blue Lass (GB) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Promoted from Day Stage 2024; Bluegrass/Old Time/Folk mix</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>Gadan (IT/IE/US) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>21:15</t>
-        </is>
-      </c>
-      <c r="F21" s="10" t="inlineStr">
-        <is>
-          <t>Celtic-Americana fusion; 3 banjo players incl. Enda Scahill (We Banjo Three)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>Hayde Bluegrass Orchestra (NO) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>21:15</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>22:30</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>2x IBMA Momentum nominees 2022; touring US regulars</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>Yellofox (NL) — Main Stage</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>22:30</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="E23" s="10" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="F23" s="10" t="inlineStr">
-        <is>
-          <t>Folk-Americana; Paul Simon/Gram Parsons influences; festival closer</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>Kids on Bluegrass Europe (Europe) — Day Stage</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>Ages 6-16; two mornings of workshops culminating in performance</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Kristy Cox Band (AU/US) — Day Stage</t>
-        </is>
-      </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="E25" s="10" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="F25" s="10" t="inlineStr">
-        <is>
-          <t>Also headlining Thu Main Stage; second chance to see them</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>That's All Folk (FR) — Day Stage</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>Local Alps trio; traditional Bluegrass + modern pop covers</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>The Sentimental Gentlemen (US) — Day Stage</t>
-        </is>
-      </c>
-      <c r="B27" s="10" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="E27" s="10" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>Also on Main Stage Fri; Sierra Ferrell's touring band</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>Tim O'Connor Trio (IE/FR) — Day Stage</t>
-        </is>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>Irishman in Aix-les-Bains; folk/Irish/blues/rock trio</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>Grace Honeywell &amp; Jeri Foreman (US/AU) — Day Stage</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="F29" s="10" t="inlineStr">
-        <is>
-          <t>Twin fiddles; folk/country; formed in UK</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>Catch the Goat (FR) — Day Stage</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>Toulouse veterans; Dawgrass style; mandocello &amp; cello</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>Shelby Means Band (US) — Day Stage</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="D31" s="10" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>Also on Sat Main Stage; entirely different set</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>Country Gongbang (KO) — Day Stage</t>
-        </is>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="F32" s="8" t="inlineStr">
-        <is>
-          <t>Also on Sat Main Stage; final chance before they fly home</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>Sweet Sally (US) — Day Stage</t>
-        </is>
-      </c>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="D33" s="10" t="inlineStr">
-        <is>
-          <t>02/08/2026</t>
-        </is>
-      </c>
-      <c r="E33" s="10" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="F33" s="10" t="inlineStr">
-        <is>
-          <t>Also on Sat Main Stage; California trio</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 1 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B34" s="16" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C34" s="16" t="inlineStr"/>
-      <c r="D34" s="16" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E34" s="16" t="inlineStr"/>
-      <c r="F34" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 2 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B35" s="16" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C35" s="16" t="inlineStr"/>
-      <c r="D35" s="16" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E35" s="16" t="inlineStr"/>
-      <c r="F35" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 3 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B36" s="16" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C36" s="16" t="inlineStr"/>
-      <c r="D36" s="16" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E36" s="16" t="inlineStr"/>
-      <c r="F36" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 4 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B37" s="16" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C37" s="16" t="inlineStr"/>
-      <c r="D37" s="16" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E37" s="16" t="inlineStr"/>
-      <c r="F37" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 5 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B38" s="16" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C38" s="16" t="inlineStr"/>
-      <c r="D38" s="16" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E38" s="16" t="inlineStr"/>
-      <c r="F38" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 6 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B39" s="16" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C39" s="16" t="inlineStr"/>
-      <c r="D39" s="16" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E39" s="16" t="inlineStr"/>
-      <c r="F39" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Offsite Concert 1 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B40" s="16" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C40" s="16" t="inlineStr"/>
-      <c r="D40" s="16" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E40" s="16" t="inlineStr"/>
-      <c r="F40" s="16" t="inlineStr">
-        <is>
-          <t>Health centre concert. FREE. Venue &amp; band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 7 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B41" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="C41" s="16" t="inlineStr"/>
-      <c r="D41" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="E41" s="16" t="inlineStr"/>
-      <c r="F41" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 8 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B42" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="C42" s="16" t="inlineStr"/>
-      <c r="D42" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="E42" s="16" t="inlineStr"/>
-      <c r="F42" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 9 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B43" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="C43" s="16" t="inlineStr"/>
-      <c r="D43" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="E43" s="16" t="inlineStr"/>
-      <c r="F43" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 10 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B44" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="C44" s="16" t="inlineStr"/>
-      <c r="D44" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="E44" s="16" t="inlineStr"/>
-      <c r="F44" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 11 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B45" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="C45" s="16" t="inlineStr"/>
-      <c r="D45" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="E45" s="16" t="inlineStr"/>
-      <c r="F45" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 12 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B46" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="C46" s="16" t="inlineStr"/>
-      <c r="D46" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="E46" s="16" t="inlineStr"/>
-      <c r="F46" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Offsite Concert 2 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B47" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="C47" s="16" t="inlineStr"/>
-      <c r="D47" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="E47" s="16" t="inlineStr"/>
-      <c r="F47" s="16" t="inlineStr">
-        <is>
-          <t>Health centre concert. FREE. Venue &amp; band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Offsite Concert 3 (TBC) — Street Festival</t>
-        </is>
-      </c>
-      <c r="B48" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="C48" s="16" t="inlineStr"/>
-      <c r="D48" s="16" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="E48" s="16" t="inlineStr"/>
-      <c r="F48" s="16" t="inlineStr">
-        <is>
-          <t>Health centre concert. FREE. Venue &amp; band TBC — check festival website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="10" t="inlineStr">
-        <is>
-          <t>Accommodation check-in (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B49" s="10" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="C49" s="10" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="D49" s="10" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="E49" s="10" t="inlineStr">
-        <is>
-          <t>School open for registration and room check-in</t>
-        </is>
-      </c>
-      <c r="F49" s="10" t="inlineStr"/>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
-        <is>
-          <t>Welcome talk &amp; drinks (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B50" s="8" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Welcome by Festival Chair and Camp Leader Gilles Rézard</t>
-        </is>
-      </c>
-      <c r="F50" s="8" t="inlineStr"/>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="10" t="inlineStr">
-        <is>
-          <t>Dinner (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B51" s="10" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="C51" s="10" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="10" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="E51" s="10" t="inlineStr"/>
-      <c r="F51" s="10" t="inlineStr"/>
-    </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="8" t="inlineStr">
-        <is>
-          <t>Breakfast (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B52" s="8" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr"/>
-      <c r="F52" s="8" t="inlineStr"/>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="10" t="inlineStr">
-        <is>
-          <t>Today's news + Instrumental classes (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B53" s="10" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="C53" s="10" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="D53" s="10" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="E53" s="10" t="inlineStr">
-        <is>
-          <t>Morning session 1 — instrumental classes</t>
-        </is>
-      </c>
-      <c r="F53" s="10" t="inlineStr"/>
-    </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="8" t="inlineStr">
-        <is>
-          <t>Break (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B54" s="8" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr"/>
-      <c r="F54" s="8" t="inlineStr"/>
-    </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="10" t="inlineStr">
-        <is>
-          <t>Instrumental classes (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B55" s="10" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="C55" s="10" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
-      <c r="D55" s="10" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="E55" s="10" t="inlineStr">
-        <is>
-          <t>Morning session 2 — instrumental classes</t>
-        </is>
-      </c>
-      <c r="F55" s="10" t="inlineStr"/>
-    </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="8" t="inlineStr">
-        <is>
-          <t>Lunch (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B56" s="8" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr"/>
-      <c r="F56" s="8" t="inlineStr"/>
-    </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="10" t="inlineStr">
-        <is>
-          <t>Wernick Method Jam: Instructions (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B57" s="10" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="C57" s="10" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="D57" s="10" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="E57" s="10" t="inlineStr">
-        <is>
-          <t>Afternoon — Wernick Method jam instructions</t>
-        </is>
-      </c>
-      <c r="F57" s="10" t="inlineStr"/>
-    </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="8" t="inlineStr">
-        <is>
-          <t>Break (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B58" s="8" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>16:30</t>
-        </is>
-      </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr"/>
-      <c r="F58" s="8" t="inlineStr"/>
-    </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="10" t="inlineStr">
-        <is>
-          <t>Optional/requested modules (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B59" s="10" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="C59" s="10" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="D59" s="10" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="E59" s="10" t="inlineStr">
-        <is>
-          <t>Requested/optional modules</t>
-        </is>
-      </c>
-      <c r="F59" s="10" t="inlineStr"/>
-    </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="8" t="inlineStr">
-        <is>
-          <t>Dinner (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B60" s="8" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>20:30</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr"/>
-      <c r="F60" s="8" t="inlineStr"/>
-    </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="10" t="inlineStr">
-        <is>
-          <t>Breakfast (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B61" s="10" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C61" s="10" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="D61" s="10" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E61" s="10" t="inlineStr"/>
-      <c r="F61" s="10" t="inlineStr"/>
-    </row>
-    <row r="62" ht="20" customHeight="1">
-      <c r="A62" s="8" t="inlineStr">
-        <is>
-          <t>Today's news + Instrumental classes (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B62" s="8" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>Morning session 1 — instrumental classes</t>
-        </is>
-      </c>
-      <c r="F62" s="8" t="inlineStr"/>
-    </row>
-    <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="10" t="inlineStr">
-        <is>
-          <t>Break (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B63" s="10" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C63" s="10" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="D63" s="10" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E63" s="10" t="inlineStr"/>
-      <c r="F63" s="10" t="inlineStr"/>
-    </row>
-    <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="8" t="inlineStr">
-        <is>
-          <t>Instrumental classes (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B64" s="8" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E64" s="8" t="inlineStr">
-        <is>
-          <t>Morning session 2 — instrumental classes</t>
-        </is>
-      </c>
-      <c r="F64" s="8" t="inlineStr"/>
-    </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="10" t="inlineStr">
-        <is>
-          <t>Lunch (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B65" s="10" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C65" s="10" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="D65" s="10" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E65" s="10" t="inlineStr"/>
-      <c r="F65" s="10" t="inlineStr"/>
-    </row>
-    <row r="66" ht="20" customHeight="1">
-      <c r="A66" s="8" t="inlineStr">
-        <is>
-          <t>Wernick Method Jam: Coached jam (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B66" s="8" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="D66" s="8" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E66" s="8" t="inlineStr">
-        <is>
-          <t>Afternoon — coached Wernick Method jam</t>
-        </is>
-      </c>
-      <c r="F66" s="8" t="inlineStr"/>
-    </row>
-    <row r="67" ht="20" customHeight="1">
-      <c r="A67" s="10" t="inlineStr">
-        <is>
-          <t>Break (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B67" s="10" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C67" s="10" t="inlineStr">
-        <is>
-          <t>16:30</t>
-        </is>
-      </c>
-      <c r="D67" s="10" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E67" s="10" t="inlineStr"/>
-      <c r="F67" s="10" t="inlineStr"/>
-    </row>
-    <row r="68" ht="20" customHeight="1">
-      <c r="A68" s="8" t="inlineStr">
-        <is>
-          <t>Concert rehearsal &amp; organisation (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B68" s="8" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="D68" s="8" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E68" s="8" t="inlineStr">
-        <is>
-          <t>Rehearsal for Thursday student concert</t>
-        </is>
-      </c>
-      <c r="F68" s="8" t="inlineStr"/>
-    </row>
-    <row r="69" ht="20" customHeight="1">
-      <c r="A69" s="10" t="inlineStr">
-        <is>
-          <t>Dinner (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B69" s="10" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="C69" s="10" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="D69" s="10" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="E69" s="10" t="inlineStr"/>
-      <c r="F69" s="10" t="inlineStr"/>
-    </row>
-    <row r="70" ht="20" customHeight="1">
-      <c r="A70" s="8" t="inlineStr">
-        <is>
-          <t>Breakfast (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B70" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="D70" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E70" s="8" t="inlineStr"/>
-      <c r="F70" s="8" t="inlineStr"/>
-    </row>
-    <row r="71" ht="20" customHeight="1">
-      <c r="A71" s="10" t="inlineStr">
-        <is>
-          <t>Today's news + Instrumental classes (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B71" s="10" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C71" s="10" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="D71" s="10" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E71" s="10" t="inlineStr">
-        <is>
-          <t>Morning session 1 — instrumental classes</t>
-        </is>
-      </c>
-      <c r="F71" s="10" t="inlineStr"/>
-    </row>
-    <row r="72" ht="20" customHeight="1">
-      <c r="A72" s="8" t="inlineStr">
-        <is>
-          <t>Break (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B72" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="D72" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E72" s="8" t="inlineStr"/>
-      <c r="F72" s="8" t="inlineStr"/>
-    </row>
-    <row r="73" ht="20" customHeight="1">
-      <c r="A73" s="10" t="inlineStr">
-        <is>
-          <t>Band labs / jams (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B73" s="10" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C73" s="10" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
-      <c r="D73" s="10" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E73" s="10" t="inlineStr">
-        <is>
-          <t>Final morning session — band labs and jams</t>
-        </is>
-      </c>
-      <c r="F73" s="10" t="inlineStr"/>
-    </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="A74" s="8" t="inlineStr">
-        <is>
-          <t>Lunch (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B74" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="D74" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E74" s="8" t="inlineStr"/>
-      <c r="F74" s="8" t="inlineStr"/>
-    </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="10" t="inlineStr">
-        <is>
-          <t>Free time (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B75" s="10" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C75" s="10" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="D75" s="10" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E75" s="10" t="inlineStr"/>
-      <c r="F75" s="10" t="inlineStr"/>
-    </row>
-    <row r="76" ht="20" customHeight="1">
-      <c r="A76" s="8" t="inlineStr">
-        <is>
-          <t>Break (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B76" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C76" s="8" t="inlineStr">
-        <is>
-          <t>16:30</t>
-        </is>
-      </c>
-      <c r="D76" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E76" s="8" t="inlineStr"/>
-      <c r="F76" s="8" t="inlineStr"/>
-    </row>
-    <row r="77" ht="20" customHeight="1">
-      <c r="A77" s="10" t="inlineStr">
-        <is>
-          <t>Head to festival site (Lycée Sainte Famille) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B77" s="10" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C77" s="10" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="D77" s="10" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E77" s="10" t="inlineStr">
-        <is>
-          <t>Move to Lycée Sainte Marie festival site</t>
-        </is>
-      </c>
-      <c r="F77" s="10" t="inlineStr"/>
-    </row>
-    <row r="78" ht="20" customHeight="1">
-      <c r="A78" s="8" t="inlineStr">
-        <is>
-          <t>Students concert — Main Stage (Festival Main Stage) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B78" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C78" s="8" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="D78" s="8" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E78" s="8" t="inlineStr">
-        <is>
-          <t>Band Labs perform on the Main Stage</t>
-        </is>
-      </c>
-      <c r="F78" s="8" t="inlineStr"/>
-    </row>
-    <row r="79" ht="20" customHeight="1">
-      <c r="A79" s="10" t="inlineStr">
-        <is>
-          <t>French teachers set — Main Stage (Festival Main Stage) — Teaching Camp</t>
-        </is>
-      </c>
-      <c r="B79" s="10" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="C79" s="10" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="D79" s="10" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="E79" s="10" t="inlineStr">
-        <is>
-          <t>French teachers perform on the Main Stage</t>
-        </is>
-      </c>
-      <c r="F79" s="10" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
adding the Street Festival
</commit_message>
<xml_diff>
--- a/LaRoche2026_Festival_Schedule.xlsx
+++ b/LaRoche2026_Festival_Schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Main Stage" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Day Stage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Street Festival" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Teaching Camp" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Stage" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day Stage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Street Festival" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teaching Camp" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,18 +60,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00B7950B"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00888888"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
       <color rgb="00B7950B"/>
       <sz val="9"/>
     </font>
@@ -130,7 +118,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
+        <fgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
     <fill>
@@ -217,10 +205,10 @@
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1932,7 +1920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2040,12 +2028,12 @@
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>TBC — Street Act 1</t>
+          <t>Watson Bridge</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">
@@ -2053,301 +2041,389 @@
           <t>Street Festival</t>
         </is>
       </c>
-      <c r="E5" s="17" t="inlineStr"/>
-      <c r="F5" s="17" t="inlineStr"/>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
+          <t>Acoustic guitar duo from the French Bluegrass scene, named after Doc Watson. Isabelle Groll and Jean-Paul Delon reinterpret American roots and Americana songwriters (Gillian Welch, Darrell Scott, Sarah Jarosz) with close vocal harmonies, joined here by Dorian Ricaux (mandolin) and Florence Chapuis (bass). Previously played La Roche in 2012 and 2016. Members: Isabelle Groll (guitar/voice), Jean-Paul Delon (guitar/voice), Dorian Ricaux (mandolin), Florence Chapuis (bass)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Wed 29 Jul</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 2</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Blue Morning Train</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>Street Festival</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr"/>
-      <c r="F6" s="17" t="inlineStr"/>
-      <c r="G6" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>French acoustic string band playing traditional American Bluegrass and roots music, touring extensively across Europe. Members: Philippe Boutet (guitar/lead vocals), Joël Amar (fiddle/vocals), Hervé Lascaux (banjo/mandolin), Isabelle Lascaux (double bass)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Wed 29 Jul</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 3</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Sweet Potato Vine</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>Street Festival</t>
         </is>
       </c>
-      <c r="E7" s="17" t="inlineStr"/>
-      <c r="F7" s="17" t="inlineStr"/>
-      <c r="G7" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>American bluegrass, old-time and folk band based in Southern France, central to the Toulouse Folk Society and the Bluegrassoulet collective. Strong vocal harmonies across traditional and modern bluegrass. Debut self-titled album includes Whiskey Down and Grey Cat on a Tennessee Farm. Members: Jake Braunecker, Léa Desplats (vocals), Maël Mesurolle (vocals/fiddle), Noémie Charmetant</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Wed 29 Jul</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 4</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Karoline &amp; the Free Folks</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Street Festival</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr"/>
-      <c r="F8" s="17" t="inlineStr"/>
-      <c r="G8" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Lyon-based Americana/country-bluegrass project led by singer-guitarist Karoline, drawing on Brandi Carlile, Trey Hensley and the Allman Brothers. Debut album Reckless Dances (2022) was followed by Blooming Haze. Performs as full amplified quartet or in stripped-back acoustic formats.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Wed 29 Jul</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 5</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Obejváci</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Street Festival</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr"/>
-      <c r="F9" s="17" t="inlineStr"/>
-      <c r="G9" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>La Brasserie Rochoise terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Wed 29 Jul</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 6</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Gospel Convicts</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Street Festival</t>
         </is>
       </c>
-      <c r="E10" s="17" t="inlineStr"/>
-      <c r="F10" s="17" t="inlineStr"/>
-      <c r="G10" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>French Bluegrass Gospel band formed in 2022 by five friends who met at a bluegrass camp, known for soaring acoustic a cappella harmonies and traditional arrangements of classic gospel and folk hymns, including Gospel Plow and Swing Low Sweet Chariot. Members: Killian De Bergh (lead vocals/guitar/banjo), Serge Aldinger (low baritone), Émilie Moretti (soprano), Marie Scheid (tenor), Mickaël Guérin (baritone)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>Wed 29 Jul</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Offsite Concert 1</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>Street Festival (Offsite)</t>
-        </is>
-      </c>
-      <c r="E11" s="17" t="inlineStr"/>
-      <c r="F11" s="17" t="inlineStr"/>
-      <c r="G11" s="16" t="inlineStr">
-        <is>
-          <t>Health centre concert. FREE. Venue &amp; band TBC.</t>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Blame the Monkey</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Street Festival</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>Italian acoustic country-bluegrass duo formed by Alejandra Del Castillo and Silvio Ferretti, both on vocals, banjo and guitar. Sets cover old and new country music, from Carter Family standards to Guy Clark and 1980s new country. The band's name nods to a playful theory that mistakes can be blamed on the chaotic 'monkeys' regulating the mind. Members: Alejandra Del Castillo (vocals/banjo/guitar), Silvio Ferretti (vocals/guitar/banjo)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>Fri 31 Jul</t>
-        </is>
-      </c>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 7</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Wed 29 Jul</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Lonesome Daze</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Street Festival</t>
         </is>
       </c>
-      <c r="E12" s="17" t="inlineStr"/>
-      <c r="F12" s="17" t="inlineStr"/>
-      <c r="G12" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Spanish acoustic bluegrass band blending traditional American bluegrass and old-time folk with a European flair. Regulars on the Spanish roots circuit and at the Al Ras Bluegrass &amp; Old-Time Festival near Barcelona.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>Fri 31 Jul</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 8</t>
-        </is>
-      </c>
-      <c r="C13" s="16" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Wed 29 Jul</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>FolKloR</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>Street Festival</t>
         </is>
       </c>
-      <c r="E13" s="17" t="inlineStr"/>
-      <c r="F13" s="17" t="inlineStr"/>
-      <c r="G13" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>French acoustic folk trio blending Irish traditional, bluegrass and jazz manouche, with a dash of power metal influence. Simon Hel (also of Carban and Broken Bow) crosses bluegrass, gypsy jazz and metal backgrounds; Perrine Bakubama brings classical, Irish and Celtic fiddle; Kor Wentemn sings and plays guitar, drawing on 60s-90s rock and folk. Members: Simon Hel (guitar), Perrine Bakubama (fiddle), Kor Wentemn (guitar/vocals)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>Fri 31 Jul</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 9</t>
-        </is>
-      </c>
-      <c r="C14" s="16" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Wed 29 Jul</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Sweet Sally</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Street Festival</t>
         </is>
       </c>
-      <c r="E14" s="17" t="inlineStr"/>
-      <c r="F14" s="17" t="inlineStr"/>
-      <c r="G14" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>La Brasserie Mino terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>Fri 31 Jul</t>
+          <t>Thu 30 Jul</t>
         </is>
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>TBC — Street Act 10</t>
+          <t>Obejváci</t>
         </is>
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>Street Festival</t>
-        </is>
-      </c>
-      <c r="E15" s="17" t="inlineStr"/>
-      <c r="F15" s="17" t="inlineStr"/>
+          <t>Street Festival (Offsite)</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
+          <t>EPSM (Établissement Public de Santé Mentale). Open to the public. FREE.</t>
         </is>
       </c>
     </row>
@@ -2359,12 +2435,12 @@
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>TBC — Street Act 11</t>
+          <t>Blue Morning Train</t>
         </is>
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
@@ -2372,98 +2448,315 @@
           <t>Street Festival</t>
         </is>
       </c>
-      <c r="E16" s="17" t="inlineStr"/>
-      <c r="F16" s="17" t="inlineStr"/>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
+          <t>French acoustic string band playing traditional American Bluegrass and roots music, touring extensively across Europe. Members: Philippe Boutet (guitar/lead vocals), Joël Amar (fiddle/vocals), Hervé Lascaux (banjo/mandolin), Isabelle Lascaux (double bass)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Fri 31 Jul</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Street Act 12</t>
-        </is>
-      </c>
-      <c r="C17" s="16" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Karoline &amp; the Free Folks</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>Street Festival</t>
         </is>
       </c>
-      <c r="E17" s="17" t="inlineStr"/>
-      <c r="F17" s="17" t="inlineStr"/>
-      <c r="G17" s="16" t="inlineStr">
-        <is>
-          <t>Bar/restaurant/café terraces around town centre. FREE. Band TBC.</t>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>Lyon-based Americana/country-bluegrass project led by singer-guitarist Karoline, drawing on Brandi Carlile, Trey Hensley and the Allman Brothers. Debut album Reckless Dances (2022) was followed by Blooming Haze. Performs as full amplified quartet or in stripped-back acoustic formats.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Fri 31 Jul</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Offsite Concert 2</t>
-        </is>
-      </c>
-      <c r="C18" s="16" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="D18" s="16" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Strawberry Moon</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Street Festival</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>French-American acoustic duo reimagining old-time, folk and bluegrass with original songwriting and rich vocal harmonies, bringing a modern feminist perspective to American roots music. Active on the European acoustic circuit, with performances at venues including The Art Café Lagny and Le Piano Vache (Paris), and at the Gloryland Festival. Members: Anaëlle Trumka (vocals/banjo/fiddle), Lucia Legnini (vocals/guitar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Fri 31 Jul</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Country GongBang</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>Street Festival</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>Le Café de la Poste terrace, town centre. Also on Day Stage and Main Stage. FREE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Fri 31 Jul</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Blame the Monkey</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Street Festival</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Italian acoustic country-bluegrass duo formed by Alejandra Del Castillo and Silvio Ferretti, both on vocals, banjo and guitar. Sets cover old and new country music, from Carter Family standards to Guy Clark and 1980s new country. The band's name nods to a playful theory that mistakes can be blamed on the chaotic 'monkeys' regulating the mind. Members: Alejandra Del Castillo (vocals/banjo/guitar), Silvio Ferretti (vocals/guitar/banjo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Fri 31 Jul</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Lonesome Daze</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>Street Festival</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>Spanish acoustic bluegrass band blending traditional American bluegrass and old-time folk with a European flair. Regulars on the Spanish roots circuit and at the Al Ras Bluegrass &amp; Old-Time Festival near Barcelona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Fri 31 Jul</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Sweet Potato Vine</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Street Festival</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>American bluegrass, old-time and folk band based in Southern France, central to the Toulouse Folk Society and the Bluegrassoulet collective. Strong vocal harmonies across traditional and modern bluegrass. Debut self-titled album includes Whiskey Down and Grey Cat on a Tennessee Farm. Members: Jake Braunecker, Léa Desplats (vocals), Maël Mesurolle (vocals/fiddle), Noémie Charmetant</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Fri 31 Jul</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Obejváci</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>Street Festival</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>La Brasserie Mino terrace, town centre. FREE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Fri 31 Jul</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Blue Lass</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>Street Festival (Offsite)</t>
         </is>
       </c>
-      <c r="E18" s="17" t="inlineStr"/>
-      <c r="F18" s="17" t="inlineStr"/>
-      <c r="G18" s="16" t="inlineStr">
-        <is>
-          <t>Health centre concert. FREE. Venue &amp; band TBC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>Fri 31 Jul</t>
-        </is>
-      </c>
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>TBC — Offsite Concert 3</t>
-        </is>
-      </c>
-      <c r="C19" s="16" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="inlineStr">
-        <is>
-          <t>Street Festival (Offsite)</t>
-        </is>
-      </c>
-      <c r="E19" s="17" t="inlineStr"/>
-      <c r="F19" s="17" t="inlineStr"/>
-      <c r="G19" s="16" t="inlineStr">
-        <is>
-          <t>Health centre concert. FREE. Venue &amp; band TBC.</t>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Le Foyer des Rocailles du Verger. Open to the public. Also on Main Stage Sunday. FREE.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed some missing bios and venues
</commit_message>
<xml_diff>
--- a/LaRoche2026_Festival_Schedule.xlsx
+++ b/LaRoche2026_Festival_Schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Main Stage" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Day Stage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Street Festival" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Teaching Camp" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Stage" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day Stage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Street Festival" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teaching Camp" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2053,7 +2053,7 @@
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Acoustic guitar duo from the French Bluegrass scene, named after Doc Watson. Isabelle Groll and Jean-Paul Delon reinterpret American roots and Americana songwriters (Gillian Welch, Darrell Scott, Sarah Jarosz) with close vocal harmonies, joined here by Dorian Ricaux (mandolin) and Florence Chapuis (bass). Previously played La Roche in 2012 and 2016. Members: Isabelle Groll (guitar/voice), Jean-Paul Delon (guitar/voice), Dorian Ricaux (mandolin), Florence Chapuis (bass)</t>
+          <t>Acoustic guitar duo from the French Bluegrass scene, named after Doc Watson. Isabelle Groll and Jean-Paul Delon reinterpret American roots and Americana songwriters (Gillian Welch, Darrell Scott, Sarah Jarosz) with close vocal harmonies, joined here by Dorian Ricaux (mandolin) and Florence Chapuis (bass). Previously played La Roche in 2012 and 2016. Members: Isabelle Groll (guitar/voice), Jean-Paul Delon (guitar/voice), Dorian Ricaux (mandolin), Florence Chapuis (bass) Efsane Kebab terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>French acoustic string band playing traditional American Bluegrass and roots music, touring extensively across Europe. Members: Philippe Boutet (guitar/lead vocals), Joël Amar (fiddle/vocals), Hervé Lascaux (banjo/mandolin), Isabelle Lascaux (double bass)</t>
+          <t>French acoustic string band playing traditional American Bluegrass and roots music, touring extensively across Europe. Members: Philippe Boutet (guitar/lead vocals), Joël Amar (fiddle/vocals), Hervé Lascaux (banjo/mandolin), Isabelle Lascaux (double bass) Noor Jahan terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>American bluegrass, old-time and folk band based in Southern France, central to the Toulouse Folk Society and the Bluegrassoulet collective. Strong vocal harmonies across traditional and modern bluegrass. Debut self-titled album includes Whiskey Down and Grey Cat on a Tennessee Farm. Members: Jake Braunecker, Léa Desplats (vocals), Maël Mesurolle (vocals/fiddle), Noémie Charmetant</t>
+          <t>American bluegrass, old-time and folk band based in Southern France, central to the Toulouse Folk Society and the Bluegrassoulet collective. Strong vocal harmonies across traditional and modern bluegrass. Debut self-titled album includes Whiskey Down and Grey Cat on a Tennessee Farm. Members: Jake Braunecker, Léa Desplats (vocals), Maël Mesurolle (vocals/fiddle), Noémie Charmetant Le Petit Café terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>Lyon-based Americana/country-bluegrass project led by singer-guitarist Karoline, drawing on Brandi Carlile, Trey Hensley and the Allman Brothers. Debut album Reckless Dances (2022) was followed by Blooming Haze. Performs as full amplified quartet or in stripped-back acoustic formats.</t>
+          <t>Lyon-based Americana/country-bluegrass project led by singer-guitarist Karoline, drawing on Brandi Carlile, Trey Hensley and the Allman Brothers. Debut album Reckless Dances (2022) was followed by Blooming Haze. Performs as full amplified quartet or in stripped-back acoustic formats. Le Bistro de la Gare terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>La Brasserie Rochoise terrace, town centre. FREE.</t>
+          <t>Rising acoustic band from South Bohemia, Czech Republic, blending American-inspired bluegrass and folk with original Czech-language songwriting. Formed in 2021, taking their name from the living room (obývák) where they first rehearsed. Debut EP Tisíc let (2024) followed by debut album Nebesák. Also showcased at the EBMA European Bluegrass Summit in Prague. Members: Kristýna Barchini (vocals/octave mandolin), Luboš Barchini (guitar/vocals), Jan Pelech (fiddle/vocals/mandolin), Petr Ježek (banjo), Štěpán Pavlíček (bass) La Brasserie Rochoise terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>French Bluegrass Gospel band formed in 2022 by five friends who met at a bluegrass camp, known for soaring acoustic a cappella harmonies and traditional arrangements of classic gospel and folk hymns, including Gospel Plow and Swing Low Sweet Chariot. Members: Killian De Bergh (lead vocals/guitar/banjo), Serge Aldinger (low baritone), Émilie Moretti (soprano), Marie Scheid (tenor), Mickaël Guérin (baritone)</t>
+          <t>French Bluegrass Gospel band formed in 2022 by five friends who met at a bluegrass camp, known for soaring acoustic a cappella harmonies and traditional arrangements of classic gospel and folk hymns, including Gospel Plow and Swing Low Sweet Chariot. Members: Killian De Bergh (lead vocals/guitar/banjo), Serge Aldinger (low baritone), Émilie Moretti (soprano), Marie Scheid (tenor), Mickaël Guérin (baritone) Le Café de la Poste / La Gavroche terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2275,7 +2275,7 @@
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>Italian acoustic country-bluegrass duo formed by Alejandra Del Castillo and Silvio Ferretti, both on vocals, banjo and guitar. Sets cover old and new country music, from Carter Family standards to Guy Clark and 1980s new country. The band's name nods to a playful theory that mistakes can be blamed on the chaotic 'monkeys' regulating the mind. Members: Alejandra Del Castillo (vocals/banjo/guitar), Silvio Ferretti (vocals/guitar/banjo)</t>
+          <t>Italian acoustic country-bluegrass duo formed by Alejandra Del Castillo and Silvio Ferretti, both on vocals, banjo and guitar. Sets cover old and new country music, from Carter Family standards to Guy Clark and 1980s new country. The band's name nods to a playful theory that mistakes can be blamed on the chaotic 'monkeys' regulating the mind. Members: Alejandra Del Castillo (vocals/banjo/guitar), Silvio Ferretti (vocals/guitar/banjo) L'Alliance terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2312,7 +2312,7 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Spanish acoustic bluegrass band blending traditional American bluegrass and old-time folk with a European flair. Regulars on the Spanish roots circuit and at the Al Ras Bluegrass &amp; Old-Time Festival near Barcelona.</t>
+          <t>Spanish acoustic bluegrass band blending traditional American bluegrass and old-time folk with a European flair. Regulars on the Spanish roots circuit and at the Al Ras Bluegrass &amp; Old-Time Festival near Barcelona. La Roche d'y Vins terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2349,7 +2349,7 @@
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>French acoustic folk trio blending Irish traditional, bluegrass and jazz manouche, with a dash of power metal influence. Simon Hel (also of Carban and Broken Bow) crosses bluegrass, gypsy jazz and metal backgrounds; Perrine Bakubama brings classical, Irish and Celtic fiddle; Kor Wentemn sings and plays guitar, drawing on 60s-90s rock and folk. Members: Simon Hel (guitar), Perrine Bakubama (fiddle), Kor Wentemn (guitar/vocals)</t>
+          <t>French acoustic folk trio blending Irish traditional, bluegrass and jazz manouche, with a dash of power metal influence. Simon Hel (also of Carban and Broken Bow) crosses bluegrass, gypsy jazz and metal backgrounds; Perrine Bakubama brings classical, Irish and Celtic fiddle; Kor Wentemn sings and plays guitar, drawing on 60s-90s rock and folk. Members: Simon Hel (guitar), Perrine Bakubama (fiddle), Kor Wentemn (guitar/vocals) Le T'cho terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
-          <t>EPSM (Établissement Public de Santé Mentale). Open to the public. FREE.</t>
+          <t>Rising acoustic band from South Bohemia, Czech Republic, blending American-inspired bluegrass and folk with original Czech-language songwriting. Formed in 2021, taking their name from the living room (obývák) where they first rehearsed. Debut EP Tisíc let (2024) followed by debut album Nebesák. Also showcased at the EBMA European Bluegrass Summit in Prague. Members: Kristýna Barchini (vocals/octave mandolin), Luboš Barchini (guitar/vocals), Jan Pelech (fiddle/vocals/mandolin), Petr Ježek (banjo), Štěpán Pavlíček (bass) EPSM (Établissement Public de Santé Mentale). Open to the public. FREE.</t>
         </is>
       </c>
     </row>
@@ -2460,7 +2460,7 @@
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
-          <t>French acoustic string band playing traditional American Bluegrass and roots music, touring extensively across Europe. Members: Philippe Boutet (guitar/lead vocals), Joël Amar (fiddle/vocals), Hervé Lascaux (banjo/mandolin), Isabelle Lascaux (double bass)</t>
+          <t>French acoustic string band playing traditional American Bluegrass and roots music, touring extensively across Europe. Members: Philippe Boutet (guitar/lead vocals), Joël Amar (fiddle/vocals), Hervé Lascaux (banjo/mandolin), Isabelle Lascaux (double bass) Bistro Tokyo terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>Lyon-based Americana/country-bluegrass project led by singer-guitarist Karoline, drawing on Brandi Carlile, Trey Hensley and the Allman Brothers. Debut album Reckless Dances (2022) was followed by Blooming Haze. Performs as full amplified quartet or in stripped-back acoustic formats.</t>
+          <t>Lyon-based Americana/country-bluegrass project led by singer-guitarist Karoline, drawing on Brandi Carlile, Trey Hensley and the Allman Brothers. Debut album Reckless Dances (2022) was followed by Blooming Haze. Performs as full amplified quartet or in stripped-back acoustic formats. Noor Jahan terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>French-American acoustic duo reimagining old-time, folk and bluegrass with original songwriting and rich vocal harmonies, bringing a modern feminist perspective to American roots music. Active on the European acoustic circuit, with performances at venues including The Art Café Lagny and Le Piano Vache (Paris), and at the Gloryland Festival. Members: Anaëlle Trumka (vocals/banjo/fiddle), Lucia Legnini (vocals/guitar)</t>
+          <t>French-American acoustic duo reimagining old-time, folk and bluegrass with original songwriting and rich vocal harmonies, bringing a modern feminist perspective to American roots music. Active on the European acoustic circuit, with performances at venues including The Art Café Lagny and Le Piano Vache (Paris), and at the Gloryland Festival. Members: Anaëlle Trumka (vocals/banjo/fiddle), Lucia Legnini (vocals/guitar) Le Petit Café terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>Italian acoustic country-bluegrass duo formed by Alejandra Del Castillo and Silvio Ferretti, both on vocals, banjo and guitar. Sets cover old and new country music, from Carter Family standards to Guy Clark and 1980s new country. The band's name nods to a playful theory that mistakes can be blamed on the chaotic 'monkeys' regulating the mind. Members: Alejandra Del Castillo (vocals/banjo/guitar), Silvio Ferretti (vocals/guitar/banjo)</t>
+          <t>Italian acoustic country-bluegrass duo formed by Alejandra Del Castillo and Silvio Ferretti, both on vocals, banjo and guitar. Sets cover old and new country music, from Carter Family standards to Guy Clark and 1980s new country. The band's name nods to a playful theory that mistakes can be blamed on the chaotic 'monkeys' regulating the mind. Members: Alejandra Del Castillo (vocals/banjo/guitar), Silvio Ferretti (vocals/guitar/banjo) La Gavroche terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>Spanish acoustic bluegrass band blending traditional American bluegrass and old-time folk with a European flair. Regulars on the Spanish roots circuit and at the Al Ras Bluegrass &amp; Old-Time Festival near Barcelona.</t>
+          <t>Spanish acoustic bluegrass band blending traditional American bluegrass and old-time folk with a European flair. Regulars on the Spanish roots circuit and at the Al Ras Bluegrass &amp; Old-Time Festival near Barcelona. Le Bistro de la Gare terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2682,7 +2682,7 @@
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>American bluegrass, old-time and folk band based in Southern France, central to the Toulouse Folk Society and the Bluegrassoulet collective. Strong vocal harmonies across traditional and modern bluegrass. Debut self-titled album includes Whiskey Down and Grey Cat on a Tennessee Farm. Members: Jake Braunecker, Léa Desplats (vocals), Maël Mesurolle (vocals/fiddle), Noémie Charmetant</t>
+          <t>American bluegrass, old-time and folk band based in Southern France, central to the Toulouse Folk Society and the Bluegrassoulet collective. Strong vocal harmonies across traditional and modern bluegrass. Debut self-titled album includes Whiskey Down and Grey Cat on a Tennessee Farm. Members: Jake Braunecker, Léa Desplats (vocals), Maël Mesurolle (vocals/fiddle), Noémie Charmetant L'Alliance terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>
@@ -2719,7 +2719,7 @@
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
-          <t>La Brasserie Mino terrace, town centre. FREE.</t>
+          <t>Rising acoustic band from South Bohemia, Czech Republic, blending American-inspired bluegrass and folk with original Czech-language songwriting. Formed in 2021, taking their name from the living room (obývák) where they first rehearsed. Debut EP Tisíc let (2024) followed by debut album Nebesák. Also showcased at the EBMA European Bluegrass Summit in Prague. Members: Kristýna Barchini (vocals/octave mandolin), Luboš Barchini (guitar/vocals), Jan Pelech (fiddle/vocals/mandolin), Petr Ježek (banjo), Štěpán Pavlíček (bass) La Brasserie Mino terrace, town centre. FREE.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added last missing bios
</commit_message>
<xml_diff>
--- a/LaRoche2026_Festival_Schedule.xlsx
+++ b/LaRoche2026_Festival_Schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Main Stage" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Day Stage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Street Festival" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Teaching Camp" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Stage" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day Stage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Street Festival" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teaching Camp" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>La Brasserie Mino terrace, town centre. FREE.</t>
+          <t>Young California trio from the CBA stable that produced Molly Tuttle and AJ Lee &amp; Blue Summit. Sophia Sparks won the 2024 Rocky Grass mandolin contest and a 2026 Berklee scholarship; Lucy Khadder is a 3-time Young Arts Award winner and Monterey Jazz Festival performer; Clare O'Grady has a background in percussion, jazz and law. Already performed at Delfest, CBA Father's Day and IBMA World of Bluegrass. EP: When the Night Falls (2025). Members: Lucy Khadder (fiddle/guitar), Sophia Sparks (mandolin/guitar), Clare O'Grady (bass) La Brasserie Mino terrace, town centre. Also on Main Stage Saturday and Day Stage Sunday. FREE.</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>Le Café de la Poste terrace, town centre. Also on Day Stage and Main Stage. FREE.</t>
+          <t>Korean Bluegrass band that has become a sensation on the US circuit since their last La Roche appearance in 2022. IBMA international band grant recipients. Standing ovations from Greyfox to the Grand Ole Opry, plus a memorable backstage jam with their hero Rhonda Vincent. Sing original compositions in Korean. Albums: We All Need Bluegrass (2025 compilation), Unknown Poets (2023). Members: Jongsu Yoon (fiddle), Yebin Kim (mandolin), Sunjae Won (guitar), Ki Ha (bass), Hyun Ho (banjo) Le Café de la Poste terrace, town centre. Also on Main Stage Saturday and Day Stage Sunday. FREE.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Le Foyer des Rocailles du Verger. Open to the public. Also on Main Stage Sunday. FREE.</t>
+          <t>UK band following the classic La Roche path: Street Festival → Day Stage (Young Talent 2024) → Main Stage 2026. Mix of Bluegrass with Old Time and Folk in both original songs and covers, reflecting a broad range of influences beyond acoustic music. EP: Skyline and Coalmines (2024). Members: Abbey Thomas (mandolin), Holly Wheeldon (fiddle/guitar), Ruth Eliza (clawhammer banjo), Esther Duerinck (fiddle), Noémie Charmetant (bass) Le Foyer des Rocailles du Verger. Open to the public. Also on Main Stage Sunday. FREE.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix dead domain links, correct street festival lineup, add venue websites
- larochebluegrass.org -> bluegrassinlaroche.org (footer, Kids on  Bluegrass Europe link)
- Fri offsite slot corrected: Tim O'Connor Trio, not Blue Lass
- L'Alliance phone number and description corrected
- Venue website links added for 9 street festival venues, surfaced as small links on band cards
- SITE_VERSION 2.4 -> 2.7
</commit_message>
<xml_diff>
--- a/LaRoche2026_Festival_Schedule.xlsx
+++ b/LaRoche2026_Festival_Schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Main Stage" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Day Stage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Street Festival" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Teaching Camp" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Stage" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day Stage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Street Festival" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teaching Camp" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2731,12 +2731,12 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Blue Lass</t>
+          <t>Tim O'Connor Trio</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IE/FR</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>UK band following the classic La Roche path: Street Festival → Day Stage (Young Talent 2024) → Main Stage 2026. Mix of Bluegrass with Old Time and Folk in both original songs and covers, reflecting a broad range of influences beyond acoustic music. EP: Skyline and Coalmines (2024). Members: Abbey Thomas (mandolin), Holly Wheeldon (fiddle/guitar), Ruth Eliza (clawhammer banjo), Esther Duerinck (fiddle), Noémie Charmetant (bass) Le Foyer des Rocailles du Verger. Open to the public. Also on Main Stage Sunday. FREE.</t>
+          <t>Irishman living locally in Aix-les-Bains; prolific singer-songwriter and 21st century troubadour. Previously played La Roche in 2009. Music crosses folk, Irish, blues and rock effortlessly. Albums: À Mery Cama (2026), Manchester St Salford Sky (2025). Members: Tim O'Connor (guitar), Bertrand Denechaud (dobro), Dave Thom (mandolin/guitar) Le Foyer des Rocailles du Verger. Open to the public. Also on Day Stage Saturday. FREE.</t>
         </is>
       </c>
     </row>

</xml_diff>